<commit_message>
Mise à jour du portfolio et du tableau de synthèse
</commit_message>
<xml_diff>
--- a/assets/EPREUVE ORALE E5 - TABLEAU DE SYNTHESE - BTS SIO 2026.xlsx
+++ b/assets/EPREUVE ORALE E5 - TABLEAU DE SYNTHESE - BTS SIO 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\data\BTS SIO 2éme Année\Support et mise à dispo SI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6DB0D60-D5DB-4C1F-84FF-D98EBC8F7484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F44EF8C-DEDD-4E68-84E3-4DD6132D92E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,6 +19,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$35</definedName>
   </definedNames>
   <calcPr calcId="101716" iterateDelta="1E-4"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -110,88 +111,88 @@
     <t>SESSION 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Site vitrine html et css
+    <t>07/11/24 - 30/11/24</t>
+  </si>
+  <si>
+    <t>NOM et prénom : MARIYATHAS ASHVIN</t>
+  </si>
+  <si>
+    <t>Centre de formation : H3 Hitema</t>
+  </si>
+  <si>
+    <t>X SLAM</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://ashvin-portfolio.dev/</t>
+  </si>
+  <si>
+    <t>N° candidat : 02248254729</t>
+  </si>
+  <si>
+    <t>25/03/25 - 19/05/25</t>
+  </si>
+  <si>
+    <t>01/09/25 - 15/12/25</t>
+  </si>
+  <si>
+    <t>15/12/25 - 15/02/26</t>
+  </si>
+  <si>
+    <t>22/09/25 - 29/09/25</t>
+  </si>
+  <si>
+    <t>16/02/26 - 16/03/26</t>
+  </si>
+  <si>
+    <t>15/01/25 - 29/08/25</t>
+  </si>
+  <si>
+    <t>03/09/25 - 06/11/25</t>
+  </si>
+  <si>
+    <t>07/11/25 - 19/12/25</t>
+  </si>
+  <si>
+    <t>15/01/25 - 29/10/25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Développer un site vitrine responsive en HTML/CSS
 (codesource, Site, CR)  </t>
   </si>
   <si>
-    <t>07/11/24 - 30/11/24</t>
-  </si>
-  <si>
-    <t>Clone Discord (php / sql / bootstrap)
+    <t>Concevoir un clone simplifié de discord avec PHP/MySQL
 (Codesource, Application, CR)</t>
   </si>
   <si>
-    <t>Projet application Java pour une billeterie
+    <t>Développer une application Java de gestion de billeterie
 (Codesource, Application, CR)</t>
   </si>
   <si>
-    <t>Mini jeu java ( Bataille Navale ) 
+    <t>Créer un mini jeu Bataille Navale en Java
 (Codesource, Application, CR)</t>
   </si>
   <si>
-    <t>TP wireframe html et css
+    <t>Réaliser une interface web responsive en HTML/CSS
 (Codesource, Site, CR)</t>
   </si>
   <si>
-    <t xml:space="preserve"> Projet Bibliothéque Laravel
+    <t>Développer une application de bibliothèque avec Laravel
  (Codesource, Application, CR)</t>
   </si>
   <si>
-    <t>Module d’apprentissage Angular – Reproduction d’une application web    (codesource, Application, CR)</t>
-  </si>
-  <si>
-    <t>Application web "QuizNova" interactive pour démontrer la maîtrise d’Angular, TypeScript et JavaScript.
+    <t>Module d’apprentissage Angular – Reproduire une application web  (codesource, Application, CR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approfondir et mettre en pratique les fondamentaux de Javascript
+(CR) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approfondir le développement front-end avec TypeScript 
+(CR) </t>
+  </si>
+  <si>
+    <t>Développer une application web "QuizNova" interactive pour démontrer la maîtrise d’Angular, TypeScript et JavaScript.
 (Codesource, Application, CR)</t>
-  </si>
-  <si>
-    <t>NOM et prénom : MARIYATHAS ASHVIN</t>
-  </si>
-  <si>
-    <t>Centre de formation : H3 Hitema</t>
-  </si>
-  <si>
-    <t>X SLAM</t>
-  </si>
-  <si>
-    <t>Adresse URL du portfolio : https://ashvin-portfolio.dev/</t>
-  </si>
-  <si>
-    <t>N° candidat : 02248254729</t>
-  </si>
-  <si>
-    <t>25/03/25 - 19/05/25</t>
-  </si>
-  <si>
-    <t>01/09/25 - 15/12/25</t>
-  </si>
-  <si>
-    <t>15/12/25 - 15/02/26</t>
-  </si>
-  <si>
-    <t>22/09/25 - 29/09/25</t>
-  </si>
-  <si>
-    <t>16/02/26 - 16/03/26</t>
-  </si>
-  <si>
-    <t>15/01/25 - 29/08/25</t>
-  </si>
-  <si>
-    <t>03/09/25 - 06/11/25</t>
-  </si>
-  <si>
-    <t>07/11/25 - 19/12/25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Module de formation TypeScript  
-(CR) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Module de formation JavaScript 
-(CR) </t>
-  </si>
-  <si>
-    <t>15/01/25 - 29/10/25</t>
   </si>
 </sst>
 </file>
@@ -734,6 +735,24 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -799,24 +818,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1142,56 +1143,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22" t="s">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="22"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="35"/>
-      <c r="H3" s="41"/>
+      <c r="A3" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="41"/>
+      <c r="H3" s="47"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="37" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="39"/>
+      <c r="A4" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="12" t="s">
         <v>8</v>
       </c>
@@ -1199,26 +1200,26 @@
         <v>15</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="31" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="33"/>
+      <c r="A5" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="39"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="35" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1241,24 +1242,24 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="306" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="21"/>
-      <c r="B7" s="30"/>
-      <c r="C7" s="43" t="s">
+      <c r="A7" s="27"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="43" t="s">
+      <c r="E7" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="43" t="s">
+      <c r="F7" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="43" t="s">
+      <c r="G7" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="45" t="s">
+      <c r="H7" s="23" t="s">
         <v>14</v>
       </c>
       <c r="I7"/>
@@ -1298,16 +1299,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="23" t="s">
+      <c r="A8" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="25"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="31"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1345,18 +1346,18 @@
       <c r="AQ8"/>
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="42" t="s">
+      <c r="A9" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>23</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="15"/>
       <c r="E9" s="15"/>
-      <c r="F9" s="44"/>
+      <c r="F9" s="22"/>
       <c r="G9" s="15"/>
-      <c r="H9" s="46"/>
+      <c r="H9" s="24"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1394,18 +1395,18 @@
       <c r="AQ9"/>
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="42" t="s">
-        <v>24</v>
+      <c r="A10" s="20" t="s">
+        <v>38</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="C10" s="15"/>
-      <c r="D10" s="44"/>
+      <c r="D10" s="22"/>
       <c r="E10" s="15"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1443,18 +1444,18 @@
       <c r="AQ10"/>
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="42" t="s">
-        <v>25</v>
+      <c r="A11" s="20" t="s">
+        <v>39</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="44"/>
+        <v>29</v>
+      </c>
+      <c r="C11" s="22"/>
       <c r="D11" s="15"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="44"/>
-      <c r="H11" s="44"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1492,18 +1493,18 @@
       <c r="AQ11"/>
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="42" t="s">
-        <v>26</v>
+      <c r="A12" s="20" t="s">
+        <v>40</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="44"/>
+        <v>30</v>
+      </c>
+      <c r="C12" s="22"/>
       <c r="D12" s="15"/>
       <c r="E12" s="15"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="44"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1541,18 +1542,18 @@
       <c r="AQ12"/>
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="42" t="s">
-        <v>27</v>
+      <c r="A13" s="20" t="s">
+        <v>41</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C13" s="15"/>
       <c r="D13" s="15"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="15"/>
-      <c r="H13" s="44"/>
+      <c r="H13" s="22"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1590,18 +1591,18 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="42" t="s">
-        <v>28</v>
+      <c r="A14" s="20" t="s">
+        <v>42</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="44"/>
+        <v>32</v>
+      </c>
+      <c r="C14" s="22"/>
       <c r="D14" s="15"/>
       <c r="E14" s="15"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="44"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1819,16 +1820,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="28"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="34"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1866,18 +1867,18 @@
       <c r="AQ19"/>
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="42" t="s">
-        <v>29</v>
+      <c r="A20" s="20" t="s">
+        <v>43</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C20" s="47"/>
+        <v>33</v>
+      </c>
+      <c r="C20" s="25"/>
       <c r="D20" s="15"/>
       <c r="E20" s="15"/>
-      <c r="F20" s="47"/>
-      <c r="G20" s="47"/>
-      <c r="H20" s="47"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="25"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1915,18 +1916,18 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="42" t="s">
-        <v>45</v>
+      <c r="A21" s="20" t="s">
+        <v>44</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C21" s="47"/>
+        <v>36</v>
+      </c>
+      <c r="C21" s="25"/>
       <c r="D21" s="15"/>
       <c r="E21" s="15"/>
-      <c r="F21" s="47"/>
-      <c r="G21" s="47"/>
-      <c r="H21" s="47"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -2189,16 +2190,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A27" s="26" t="s">
+      <c r="A27" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="28"/>
+      <c r="B27" s="33"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="34"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2236,18 +2237,18 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="42" t="s">
-        <v>44</v>
+      <c r="A28" s="20" t="s">
+        <v>45</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28" s="47"/>
+        <v>34</v>
+      </c>
+      <c r="C28" s="25"/>
       <c r="D28" s="15"/>
       <c r="E28" s="15"/>
-      <c r="F28" s="47"/>
-      <c r="G28" s="47"/>
-      <c r="H28" s="47"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2285,18 +2286,18 @@
       <c r="AQ28"/>
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="42" t="s">
-        <v>30</v>
+      <c r="A29" s="20" t="s">
+        <v>46</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C29" s="47"/>
-      <c r="D29" s="47"/>
+        <v>35</v>
+      </c>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
       <c r="E29" s="15"/>
-      <c r="F29" s="47"/>
-      <c r="G29" s="47"/>
-      <c r="H29" s="47"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="25"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>

</xml_diff>